<commit_message>
Importa 3 estradas novas em Tucano da última correção da bancada
3 estradas realmente novas (~5,5km) das 278 no export — o resto já eram
cadastradas ou remoções já aplicadas antes. Bancada unificada também ganha
listas separadas com cabeçalho colorido pra "traçados errados", "estradas
já cadastradas" e "estradas novas desenhadas agora" — pedido do usuário
pra não misturar tudo numa lista só.
</commit_message>
<xml_diff>
--- a/FAZENDA_TUCANO_distancias.xlsx
+++ b/FAZENDA_TUCANO_distancias.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76ED30C4-DCCE-4B1A-AFD5-C9F75276A5B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6127F424-DF2F-4FDD-A9A9-DD8F78712100}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="108">
   <si>
     <t>FAZENDA TUCANO — distância dos talhões até a sede</t>
   </si>
@@ -240,6 +240,9 @@
     <t>T-04</t>
   </si>
   <si>
+    <t>T-06B</t>
+  </si>
+  <si>
     <t>T-07</t>
   </si>
   <si>
@@ -261,6 +264,9 @@
     <t>T-02</t>
   </si>
   <si>
+    <t>T-06C</t>
+  </si>
+  <si>
     <t>T-01</t>
   </si>
   <si>
@@ -277,12 +283,6 @@
   </si>
   <si>
     <t>sem estrada até este talhão</t>
-  </si>
-  <si>
-    <t>T-06B</t>
-  </si>
-  <si>
-    <t>T-06C</t>
   </si>
   <si>
     <t>T-40C</t>
@@ -1961,15 +1961,15 @@
         <v>9361</v>
       </c>
       <c r="G37" s="8">
-        <f t="shared" ref="G37:G69" si="3">D37/1000</f>
+        <f t="shared" ref="G37:G71" si="3">D37/1000</f>
         <v>19.047999999999998</v>
       </c>
       <c r="H37" s="8">
-        <f t="shared" ref="H37:H69" si="4">E37/1000</f>
+        <f t="shared" ref="H37:H71" si="4">E37/1000</f>
         <v>16.024000000000001</v>
       </c>
       <c r="I37" s="9">
-        <f t="shared" ref="I37:I69" si="5">IFERROR(D37/F37,"")</f>
+        <f t="shared" ref="I37:I71" si="5">IFERROR(D37/F37,"")</f>
         <v>2.0348253391731652</v>
       </c>
       <c r="J37" s="10"/>
@@ -2447,7 +2447,7 @@
         <v>7672</v>
       </c>
       <c r="D52" s="14">
-        <v>11835</v>
+        <v>12406</v>
       </c>
       <c r="E52" s="14">
         <v>8224</v>
@@ -2457,7 +2457,7 @@
       </c>
       <c r="G52" s="15">
         <f t="shared" si="3"/>
-        <v>11.835000000000001</v>
+        <v>12.406000000000001</v>
       </c>
       <c r="H52" s="15">
         <f t="shared" si="4"/>
@@ -2465,7 +2465,7 @@
       </c>
       <c r="I52" s="16">
         <f t="shared" si="5"/>
-        <v>2.0072930800542741</v>
+        <v>2.1041383989145181</v>
       </c>
       <c r="J52" s="17"/>
     </row>
@@ -2738,31 +2738,31 @@
         <v>68</v>
       </c>
       <c r="B61" s="19">
-        <v>93.41</v>
+        <v>40.44</v>
       </c>
       <c r="C61" s="20">
-        <v>4212</v>
+        <v>2957</v>
       </c>
       <c r="D61" s="21">
-        <v>9600</v>
+        <v>9658</v>
       </c>
       <c r="E61" s="21">
-        <v>8252</v>
+        <v>8939</v>
       </c>
       <c r="F61" s="21">
-        <v>539</v>
+        <v>2698</v>
       </c>
       <c r="G61" s="22">
         <f t="shared" si="3"/>
-        <v>9.6</v>
+        <v>9.6579999999999995</v>
       </c>
       <c r="H61" s="22">
         <f t="shared" si="4"/>
-        <v>8.2520000000000007</v>
+        <v>8.9390000000000001</v>
       </c>
       <c r="I61" s="23">
         <f t="shared" si="5"/>
-        <v>17.810760667903526</v>
+        <v>3.5796886582653817</v>
       </c>
       <c r="J61" s="24"/>
     </row>
@@ -2771,130 +2771,130 @@
         <v>69</v>
       </c>
       <c r="B62" s="19">
-        <v>30.12</v>
+        <v>93.41</v>
       </c>
       <c r="C62" s="20">
-        <v>2592</v>
+        <v>4212</v>
       </c>
       <c r="D62" s="21">
-        <v>9450</v>
+        <v>9600</v>
       </c>
       <c r="E62" s="21">
-        <v>8286</v>
+        <v>8252</v>
       </c>
       <c r="F62" s="21">
-        <v>929</v>
+        <v>539</v>
       </c>
       <c r="G62" s="22">
         <f t="shared" si="3"/>
-        <v>9.4499999999999993</v>
+        <v>9.6</v>
       </c>
       <c r="H62" s="22">
         <f t="shared" si="4"/>
-        <v>8.2859999999999996</v>
+        <v>8.2520000000000007</v>
       </c>
       <c r="I62" s="23">
         <f t="shared" si="5"/>
+        <v>17.810760667903526</v>
+      </c>
+      <c r="J62" s="24"/>
+    </row>
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A63" s="18" t="s">
+        <v>70</v>
+      </c>
+      <c r="B63" s="19">
+        <v>30.12</v>
+      </c>
+      <c r="C63" s="20">
+        <v>2592</v>
+      </c>
+      <c r="D63" s="21">
+        <v>9450</v>
+      </c>
+      <c r="E63" s="21">
+        <v>8286</v>
+      </c>
+      <c r="F63" s="21">
+        <v>929</v>
+      </c>
+      <c r="G63" s="22">
+        <f t="shared" si="3"/>
+        <v>9.4499999999999993</v>
+      </c>
+      <c r="H63" s="22">
+        <f t="shared" si="4"/>
+        <v>8.2859999999999996</v>
+      </c>
+      <c r="I63" s="23">
+        <f t="shared" si="5"/>
         <v>10.172228202368137</v>
       </c>
-      <c r="J62" s="24"/>
-    </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A63" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="B63" s="5">
+      <c r="J63" s="24"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A64" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B64" s="12">
         <v>46.34</v>
       </c>
-      <c r="C63" s="6">
+      <c r="C64" s="13">
         <v>2872</v>
       </c>
-      <c r="D63" s="7">
+      <c r="D64" s="14">
         <v>8982</v>
       </c>
-      <c r="E63" s="7">
+      <c r="E64" s="14">
         <v>7133</v>
       </c>
-      <c r="F63" s="7">
+      <c r="F64" s="14">
         <v>5202</v>
       </c>
-      <c r="G63" s="8">
+      <c r="G64" s="15">
         <f t="shared" si="3"/>
         <v>8.9819999999999993</v>
       </c>
-      <c r="H63" s="8">
+      <c r="H64" s="15">
         <f t="shared" si="4"/>
         <v>7.133</v>
       </c>
-      <c r="I63" s="9">
+      <c r="I64" s="16">
         <f t="shared" si="5"/>
         <v>1.726643598615917</v>
       </c>
-      <c r="J63" s="10"/>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A64" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="B64" s="19">
-        <v>286.07</v>
-      </c>
-      <c r="C64" s="20">
-        <v>6866</v>
-      </c>
-      <c r="D64" s="21">
-        <v>8739</v>
-      </c>
-      <c r="E64" s="21">
-        <v>5244</v>
-      </c>
-      <c r="F64" s="21">
-        <v>2661</v>
-      </c>
-      <c r="G64" s="22">
-        <f t="shared" si="3"/>
-        <v>8.7390000000000008</v>
-      </c>
-      <c r="H64" s="22">
-        <f t="shared" si="4"/>
-        <v>5.2439999999999998</v>
-      </c>
-      <c r="I64" s="23">
-        <f t="shared" si="5"/>
-        <v>3.2841037204058625</v>
-      </c>
-      <c r="J64" s="24"/>
+      <c r="J64" s="17"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="18" t="s">
         <v>72</v>
       </c>
       <c r="B65" s="19">
-        <v>39.74</v>
+        <v>286.07</v>
       </c>
       <c r="C65" s="20">
-        <v>3355</v>
+        <v>6866</v>
       </c>
       <c r="D65" s="21">
-        <v>8286</v>
+        <v>8739</v>
       </c>
       <c r="E65" s="21">
-        <v>7283</v>
+        <v>5244</v>
       </c>
       <c r="F65" s="21">
-        <v>1816</v>
+        <v>2661</v>
       </c>
       <c r="G65" s="22">
         <f t="shared" si="3"/>
-        <v>8.2859999999999996</v>
+        <v>8.7390000000000008</v>
       </c>
       <c r="H65" s="22">
         <f t="shared" si="4"/>
-        <v>7.2830000000000004</v>
+        <v>5.2439999999999998</v>
       </c>
       <c r="I65" s="23">
         <f t="shared" si="5"/>
-        <v>4.5627753303964758</v>
+        <v>3.2841037204058625</v>
       </c>
       <c r="J65" s="24"/>
     </row>
@@ -2903,19 +2903,19 @@
         <v>73</v>
       </c>
       <c r="B66" s="19">
-        <v>72.52</v>
+        <v>39.74</v>
       </c>
       <c r="C66" s="20">
-        <v>3558</v>
+        <v>3355</v>
       </c>
       <c r="D66" s="21">
         <v>8286</v>
       </c>
       <c r="E66" s="21">
-        <v>6044</v>
+        <v>7283</v>
       </c>
       <c r="F66" s="21">
-        <v>1840</v>
+        <v>1816</v>
       </c>
       <c r="G66" s="22">
         <f t="shared" si="3"/>
@@ -2923,11 +2923,11 @@
       </c>
       <c r="H66" s="22">
         <f t="shared" si="4"/>
-        <v>6.0439999999999996</v>
+        <v>7.2830000000000004</v>
       </c>
       <c r="I66" s="23">
         <f t="shared" si="5"/>
-        <v>4.5032608695652172</v>
+        <v>4.5627753303964758</v>
       </c>
       <c r="J66" s="24"/>
     </row>
@@ -2936,31 +2936,31 @@
         <v>74</v>
       </c>
       <c r="B67" s="19">
-        <v>159.81</v>
+        <v>72.52</v>
       </c>
       <c r="C67" s="20">
-        <v>5989</v>
+        <v>3558</v>
       </c>
       <c r="D67" s="21">
-        <v>5271</v>
+        <v>8286</v>
       </c>
       <c r="E67" s="21">
-        <v>3243</v>
+        <v>6044</v>
       </c>
       <c r="F67" s="21">
-        <v>623</v>
+        <v>1840</v>
       </c>
       <c r="G67" s="22">
         <f t="shared" si="3"/>
-        <v>5.2709999999999999</v>
+        <v>8.2859999999999996</v>
       </c>
       <c r="H67" s="22">
         <f t="shared" si="4"/>
-        <v>3.2429999999999999</v>
+        <v>6.0439999999999996</v>
       </c>
       <c r="I67" s="23">
         <f t="shared" si="5"/>
-        <v>8.4606741573033712</v>
+        <v>4.5032608695652172</v>
       </c>
       <c r="J67" s="24"/>
     </row>
@@ -2969,161 +2969,163 @@
         <v>75</v>
       </c>
       <c r="B68" s="19">
-        <v>110.29</v>
+        <v>159.81</v>
       </c>
       <c r="C68" s="20">
-        <v>5351</v>
+        <v>5989</v>
       </c>
       <c r="D68" s="21">
-        <v>4395</v>
+        <v>5271</v>
       </c>
       <c r="E68" s="21">
-        <v>616</v>
+        <v>3243</v>
       </c>
       <c r="F68" s="21">
-        <v>172</v>
+        <v>623</v>
       </c>
       <c r="G68" s="22">
         <f t="shared" si="3"/>
-        <v>4.3949999999999996</v>
+        <v>5.2709999999999999</v>
       </c>
       <c r="H68" s="22">
         <f t="shared" si="4"/>
-        <v>0.61599999999999999</v>
+        <v>3.2429999999999999</v>
       </c>
       <c r="I68" s="23">
         <f t="shared" si="5"/>
-        <v>25.552325581395348</v>
+        <v>8.4606741573033712</v>
       </c>
       <c r="J68" s="24"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A69" s="18" t="s">
+      <c r="A69" s="4" t="s">
         <v>76</v>
       </c>
-      <c r="B69" s="19">
-        <v>29.65</v>
-      </c>
-      <c r="C69" s="20">
-        <v>2527</v>
-      </c>
-      <c r="D69" s="21">
-        <v>1536</v>
-      </c>
-      <c r="E69" s="21">
-        <v>266</v>
-      </c>
-      <c r="F69" s="21">
-        <v>250</v>
-      </c>
-      <c r="G69" s="22">
+      <c r="B69" s="5">
+        <v>36.46</v>
+      </c>
+      <c r="C69" s="6">
+        <v>2605</v>
+      </c>
+      <c r="D69" s="7">
+        <v>4420</v>
+      </c>
+      <c r="E69" s="7">
+        <v>4380</v>
+      </c>
+      <c r="F69" s="7">
+        <v>3603</v>
+      </c>
+      <c r="G69" s="8">
         <f t="shared" si="3"/>
-        <v>1.536</v>
-      </c>
-      <c r="H69" s="22">
+        <v>4.42</v>
+      </c>
+      <c r="H69" s="8">
         <f t="shared" si="4"/>
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="I69" s="23">
+        <v>4.38</v>
+      </c>
+      <c r="I69" s="9">
         <f t="shared" si="5"/>
-        <v>6.1440000000000001</v>
-      </c>
-      <c r="J69" s="24"/>
+        <v>1.2267554815431585</v>
+      </c>
+      <c r="J69" s="10"/>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="18" t="s">
         <v>77</v>
       </c>
       <c r="B70" s="19">
-        <v>33.869999999999997</v>
+        <v>110.29</v>
       </c>
       <c r="C70" s="20">
-        <v>2696</v>
-      </c>
-      <c r="D70" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="E70" s="25" t="s">
-        <v>78</v>
+        <v>5351</v>
+      </c>
+      <c r="D70" s="21">
+        <v>4395</v>
+      </c>
+      <c r="E70" s="21">
+        <v>616</v>
       </c>
       <c r="F70" s="21">
-        <v>3966</v>
-      </c>
-      <c r="G70" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="H70" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="I70" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="J70" s="28" t="s">
-        <v>80</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="G70" s="22">
+        <f t="shared" si="3"/>
+        <v>4.3949999999999996</v>
+      </c>
+      <c r="H70" s="22">
+        <f t="shared" si="4"/>
+        <v>0.61599999999999999</v>
+      </c>
+      <c r="I70" s="23">
+        <f t="shared" si="5"/>
+        <v>25.552325581395348</v>
+      </c>
+      <c r="J70" s="24"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="18" t="s">
-        <v>81</v>
+        <v>78</v>
       </c>
       <c r="B71" s="19">
-        <v>40.44</v>
+        <v>29.65</v>
       </c>
       <c r="C71" s="20">
-        <v>2957</v>
-      </c>
-      <c r="D71" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="E71" s="25" t="s">
-        <v>78</v>
+        <v>2527</v>
+      </c>
+      <c r="D71" s="21">
+        <v>1536</v>
+      </c>
+      <c r="E71" s="21">
+        <v>266</v>
       </c>
       <c r="F71" s="21">
-        <v>2698</v>
-      </c>
-      <c r="G71" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="H71" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="I71" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="J71" s="28" t="s">
-        <v>80</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="G71" s="22">
+        <f t="shared" si="3"/>
+        <v>1.536</v>
+      </c>
+      <c r="H71" s="22">
+        <f t="shared" si="4"/>
+        <v>0.26600000000000001</v>
+      </c>
+      <c r="I71" s="23">
+        <f t="shared" si="5"/>
+        <v>6.1440000000000001</v>
+      </c>
+      <c r="J71" s="24"/>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="B72" s="19">
+        <v>33.869999999999997</v>
+      </c>
+      <c r="C72" s="20">
+        <v>2696</v>
+      </c>
+      <c r="D72" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="E72" s="25" t="s">
+        <v>80</v>
+      </c>
+      <c r="F72" s="21">
+        <v>3966</v>
+      </c>
+      <c r="G72" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="H72" s="26" t="s">
+        <v>81</v>
+      </c>
+      <c r="I72" s="27" t="s">
+        <v>81</v>
+      </c>
+      <c r="J72" s="28" t="s">
         <v>82</v>
-      </c>
-      <c r="B72" s="19">
-        <v>36.46</v>
-      </c>
-      <c r="C72" s="20">
-        <v>2605</v>
-      </c>
-      <c r="D72" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="E72" s="25" t="s">
-        <v>78</v>
-      </c>
-      <c r="F72" s="21">
-        <v>3603</v>
-      </c>
-      <c r="G72" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="H72" s="26" t="s">
-        <v>79</v>
-      </c>
-      <c r="I72" s="27" t="s">
-        <v>79</v>
-      </c>
-      <c r="J72" s="28" t="s">
-        <v>80</v>
       </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
@@ -3137,25 +3139,25 @@
         <v>2528</v>
       </c>
       <c r="D73" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E73" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F73" s="21">
         <v>13714</v>
       </c>
       <c r="G73" s="26" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H73" s="26" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I73" s="27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J73" s="28" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
@@ -3169,25 +3171,25 @@
         <v>1056</v>
       </c>
       <c r="D74" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="E74" s="25" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F74" s="21">
         <v>3969</v>
       </c>
       <c r="G74" s="26" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="H74" s="26" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="I74" s="27" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="J74" s="28" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
@@ -3208,7 +3210,7 @@
       </c>
       <c r="I76" s="33">
         <f>IFERROR(AVERAGE(I5:I74),"")</f>
-        <v>3.7325692574407903</v>
+        <v>3.6943327043629872</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
T-05D e T-CON (Tucano) saem de "sem acesso" via ponto de exceção confirmado
Regime de exceção pontual: usuário identificou, olhando a imagem de
satélite, que o acesso real desses dois talhões começa perto de T-06A,
num ponto que já está a poucos metros de uma estrada digitalizada. A
distância agora é medida a partir desse ponto (7,71 km até a sede),
com aviso visível na ficha explicando que não há estrada traçada até o
próprio talhão.

Cache-busting do dados_mapa.js.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FAZENDA_TUCANO_distancias.xlsx
+++ b/FAZENDA_TUCANO_distancias.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhao\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhoes-distancias\saidas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ED1BAE8-6B5C-4E0C-8E3F-D25C1F5907AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B788502D-BC5B-4954-BDCD-B4033741965B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2232" yWindow="2232" windowWidth="14100" windowHeight="9792" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Distâncias" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="108">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="108">
   <si>
     <t>FAZENDA TUCANO — distância dos talhões até a sede</t>
   </si>
@@ -243,6 +243,12 @@
     <t>T-16</t>
   </si>
   <si>
+    <t>T-05D</t>
+  </si>
+  <si>
+    <t>T-CON</t>
+  </si>
+  <si>
     <t>T-06A</t>
   </si>
   <si>
@@ -273,7 +279,7 @@
     <t>T-10</t>
   </si>
   <si>
-    <t>T-05D</t>
+    <t>T-40C</t>
   </si>
   <si>
     <t>sem acesso</t>
@@ -283,12 +289,6 @@
   </si>
   <si>
     <t>sem estrada até este talhão</t>
-  </si>
-  <si>
-    <t>T-40C</t>
-  </si>
-  <si>
-    <t>T-CON</t>
   </si>
   <si>
     <t>TOTAL / MÁXIMO</t>
@@ -1961,15 +1961,15 @@
         <v>10413</v>
       </c>
       <c r="G37" s="8">
-        <f t="shared" ref="G37:G71" si="3">D37/1000</f>
+        <f t="shared" ref="G37:G73" si="3">D37/1000</f>
         <v>18.309999999999999</v>
       </c>
       <c r="H37" s="8">
-        <f t="shared" ref="H37:H71" si="4">E37/1000</f>
+        <f t="shared" ref="H37:H73" si="4">E37/1000</f>
         <v>17.29</v>
       </c>
       <c r="I37" s="9">
-        <f t="shared" ref="I37:I71" si="5">IFERROR(D37/F37,"")</f>
+        <f t="shared" ref="I37:I73" si="5">IFERROR(D37/F37,"")</f>
         <v>1.7583789493901854</v>
       </c>
       <c r="J37" s="10"/>
@@ -2767,101 +2767,101 @@
       <c r="J61" s="10"/>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A62" s="18" t="s">
+      <c r="A62" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="B62" s="19">
-        <v>39.74</v>
-      </c>
-      <c r="C62" s="20">
-        <v>3355</v>
-      </c>
-      <c r="D62" s="21">
-        <v>7579</v>
-      </c>
-      <c r="E62" s="21">
-        <v>6617</v>
-      </c>
-      <c r="F62" s="21">
-        <v>1816</v>
-      </c>
-      <c r="G62" s="22">
-        <f t="shared" si="3"/>
-        <v>7.5789999999999997</v>
-      </c>
-      <c r="H62" s="22">
-        <f t="shared" si="4"/>
-        <v>6.617</v>
-      </c>
-      <c r="I62" s="23">
-        <f t="shared" si="5"/>
-        <v>4.1734581497797354</v>
-      </c>
-      <c r="J62" s="24"/>
+      <c r="B62" s="12">
+        <v>33.869999999999997</v>
+      </c>
+      <c r="C62" s="13">
+        <v>2696</v>
+      </c>
+      <c r="D62" s="14">
+        <v>7715</v>
+      </c>
+      <c r="E62" s="14">
+        <v>7715</v>
+      </c>
+      <c r="F62" s="14">
+        <v>3966</v>
+      </c>
+      <c r="G62" s="15">
+        <f t="shared" si="3"/>
+        <v>7.7149999999999999</v>
+      </c>
+      <c r="H62" s="15">
+        <f t="shared" si="4"/>
+        <v>7.7149999999999999</v>
+      </c>
+      <c r="I62" s="16">
+        <f t="shared" si="5"/>
+        <v>1.9452849218356025</v>
+      </c>
+      <c r="J62" s="17"/>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A63" s="18" t="s">
+      <c r="A63" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="B63" s="19">
-        <v>72.52</v>
-      </c>
-      <c r="C63" s="20">
-        <v>3558</v>
-      </c>
-      <c r="D63" s="21">
-        <v>7432</v>
-      </c>
-      <c r="E63" s="21">
-        <v>6033</v>
-      </c>
-      <c r="F63" s="21">
-        <v>1840</v>
-      </c>
-      <c r="G63" s="22">
-        <f t="shared" si="3"/>
-        <v>7.4320000000000004</v>
-      </c>
-      <c r="H63" s="22">
-        <f t="shared" si="4"/>
-        <v>6.0330000000000004</v>
-      </c>
-      <c r="I63" s="23">
-        <f t="shared" si="5"/>
-        <v>4.0391304347826091</v>
-      </c>
-      <c r="J63" s="24"/>
+      <c r="B63" s="5">
+        <v>3.24</v>
+      </c>
+      <c r="C63" s="6">
+        <v>1056</v>
+      </c>
+      <c r="D63" s="7">
+        <v>7715</v>
+      </c>
+      <c r="E63" s="7">
+        <v>7715</v>
+      </c>
+      <c r="F63" s="7">
+        <v>3969</v>
+      </c>
+      <c r="G63" s="8">
+        <f t="shared" si="3"/>
+        <v>7.7149999999999999</v>
+      </c>
+      <c r="H63" s="8">
+        <f t="shared" si="4"/>
+        <v>7.7149999999999999</v>
+      </c>
+      <c r="I63" s="9">
+        <f t="shared" si="5"/>
+        <v>1.9438145628621819</v>
+      </c>
+      <c r="J63" s="10"/>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="18" t="s">
         <v>71</v>
       </c>
       <c r="B64" s="19">
-        <v>93.41</v>
+        <v>39.74</v>
       </c>
       <c r="C64" s="20">
-        <v>4212</v>
+        <v>3355</v>
       </c>
       <c r="D64" s="21">
-        <v>6651</v>
+        <v>7579</v>
       </c>
       <c r="E64" s="21">
-        <v>5303</v>
+        <v>6617</v>
       </c>
       <c r="F64" s="21">
-        <v>539</v>
+        <v>1816</v>
       </c>
       <c r="G64" s="22">
         <f t="shared" si="3"/>
-        <v>6.6509999999999998</v>
+        <v>7.5789999999999997</v>
       </c>
       <c r="H64" s="22">
         <f t="shared" si="4"/>
-        <v>5.3029999999999999</v>
+        <v>6.617</v>
       </c>
       <c r="I64" s="23">
         <f t="shared" si="5"/>
-        <v>12.339517625231911</v>
+        <v>4.1734581497797354</v>
       </c>
       <c r="J64" s="24"/>
     </row>
@@ -2870,31 +2870,31 @@
         <v>72</v>
       </c>
       <c r="B65" s="19">
-        <v>30.12</v>
+        <v>72.52</v>
       </c>
       <c r="C65" s="20">
-        <v>2592</v>
+        <v>3558</v>
       </c>
       <c r="D65" s="21">
-        <v>6617</v>
+        <v>7432</v>
       </c>
       <c r="E65" s="21">
-        <v>5688</v>
+        <v>6033</v>
       </c>
       <c r="F65" s="21">
-        <v>929</v>
+        <v>1840</v>
       </c>
       <c r="G65" s="22">
         <f t="shared" si="3"/>
-        <v>6.617</v>
+        <v>7.4320000000000004</v>
       </c>
       <c r="H65" s="22">
         <f t="shared" si="4"/>
-        <v>5.6879999999999997</v>
+        <v>6.0330000000000004</v>
       </c>
       <c r="I65" s="23">
         <f t="shared" si="5"/>
-        <v>7.1227125941872984</v>
+        <v>4.0391304347826091</v>
       </c>
       <c r="J65" s="24"/>
     </row>
@@ -2903,31 +2903,31 @@
         <v>73</v>
       </c>
       <c r="B66" s="19">
-        <v>159.81</v>
+        <v>93.41</v>
       </c>
       <c r="C66" s="20">
-        <v>5989</v>
+        <v>4212</v>
       </c>
       <c r="D66" s="21">
-        <v>6061</v>
+        <v>6651</v>
       </c>
       <c r="E66" s="21">
-        <v>3243</v>
+        <v>5303</v>
       </c>
       <c r="F66" s="21">
-        <v>623</v>
+        <v>539</v>
       </c>
       <c r="G66" s="22">
         <f t="shared" si="3"/>
-        <v>6.0609999999999999</v>
+        <v>6.6509999999999998</v>
       </c>
       <c r="H66" s="22">
         <f t="shared" si="4"/>
-        <v>3.2429999999999999</v>
+        <v>5.3029999999999999</v>
       </c>
       <c r="I66" s="23">
         <f t="shared" si="5"/>
-        <v>9.728731942215088</v>
+        <v>12.339517625231911</v>
       </c>
       <c r="J66" s="24"/>
     </row>
@@ -2936,31 +2936,31 @@
         <v>74</v>
       </c>
       <c r="B67" s="19">
-        <v>226.37</v>
+        <v>30.12</v>
       </c>
       <c r="C67" s="20">
-        <v>7413</v>
+        <v>2592</v>
       </c>
       <c r="D67" s="21">
-        <v>6005</v>
+        <v>6617</v>
       </c>
       <c r="E67" s="21">
-        <v>3122</v>
+        <v>5688</v>
       </c>
       <c r="F67" s="21">
-        <v>554</v>
+        <v>929</v>
       </c>
       <c r="G67" s="22">
         <f t="shared" si="3"/>
-        <v>6.0049999999999999</v>
+        <v>6.617</v>
       </c>
       <c r="H67" s="22">
         <f t="shared" si="4"/>
-        <v>3.1219999999999999</v>
+        <v>5.6879999999999997</v>
       </c>
       <c r="I67" s="23">
         <f t="shared" si="5"/>
-        <v>10.839350180505415</v>
+        <v>7.1227125941872984</v>
       </c>
       <c r="J67" s="24"/>
     </row>
@@ -2969,227 +2969,229 @@
         <v>75</v>
       </c>
       <c r="B68" s="19">
-        <v>127.8</v>
+        <v>159.81</v>
       </c>
       <c r="C68" s="20">
-        <v>5228</v>
+        <v>5989</v>
       </c>
       <c r="D68" s="21">
-        <v>5303</v>
+        <v>6061</v>
       </c>
       <c r="E68" s="21">
-        <v>1483</v>
+        <v>3243</v>
       </c>
       <c r="F68" s="21">
-        <v>289</v>
+        <v>623</v>
       </c>
       <c r="G68" s="22">
         <f t="shared" si="3"/>
-        <v>5.3029999999999999</v>
+        <v>6.0609999999999999</v>
       </c>
       <c r="H68" s="22">
         <f t="shared" si="4"/>
-        <v>1.4830000000000001</v>
+        <v>3.2429999999999999</v>
       </c>
       <c r="I68" s="23">
         <f t="shared" si="5"/>
-        <v>18.349480968858131</v>
+        <v>9.728731942215088</v>
       </c>
       <c r="J68" s="24"/>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
+      <c r="A69" s="18" t="s">
         <v>76</v>
       </c>
-      <c r="B69" s="5">
-        <v>36.46</v>
-      </c>
-      <c r="C69" s="6">
-        <v>2605</v>
-      </c>
-      <c r="D69" s="7">
-        <v>4420</v>
-      </c>
-      <c r="E69" s="7">
-        <v>4380</v>
-      </c>
-      <c r="F69" s="7">
-        <v>3603</v>
-      </c>
-      <c r="G69" s="8">
-        <f t="shared" si="3"/>
-        <v>4.42</v>
-      </c>
-      <c r="H69" s="8">
-        <f t="shared" si="4"/>
-        <v>4.38</v>
-      </c>
-      <c r="I69" s="9">
-        <f t="shared" si="5"/>
-        <v>1.2267554815431585</v>
-      </c>
-      <c r="J69" s="10"/>
+      <c r="B69" s="19">
+        <v>226.37</v>
+      </c>
+      <c r="C69" s="20">
+        <v>7413</v>
+      </c>
+      <c r="D69" s="21">
+        <v>6005</v>
+      </c>
+      <c r="E69" s="21">
+        <v>3122</v>
+      </c>
+      <c r="F69" s="21">
+        <v>554</v>
+      </c>
+      <c r="G69" s="22">
+        <f t="shared" si="3"/>
+        <v>6.0049999999999999</v>
+      </c>
+      <c r="H69" s="22">
+        <f t="shared" si="4"/>
+        <v>3.1219999999999999</v>
+      </c>
+      <c r="I69" s="23">
+        <f t="shared" si="5"/>
+        <v>10.839350180505415</v>
+      </c>
+      <c r="J69" s="24"/>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="18" t="s">
         <v>77</v>
       </c>
       <c r="B70" s="19">
-        <v>110.29</v>
+        <v>127.8</v>
       </c>
       <c r="C70" s="20">
-        <v>5351</v>
+        <v>5228</v>
       </c>
       <c r="D70" s="21">
-        <v>4395</v>
+        <v>5303</v>
       </c>
       <c r="E70" s="21">
-        <v>616</v>
+        <v>1483</v>
       </c>
       <c r="F70" s="21">
-        <v>172</v>
+        <v>289</v>
       </c>
       <c r="G70" s="22">
         <f t="shared" si="3"/>
-        <v>4.3949999999999996</v>
+        <v>5.3029999999999999</v>
       </c>
       <c r="H70" s="22">
         <f t="shared" si="4"/>
-        <v>0.61599999999999999</v>
+        <v>1.4830000000000001</v>
       </c>
       <c r="I70" s="23">
         <f t="shared" si="5"/>
-        <v>25.552325581395348</v>
+        <v>18.349480968858131</v>
       </c>
       <c r="J70" s="24"/>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A71" s="18" t="s">
+      <c r="A71" s="4" t="s">
         <v>78</v>
       </c>
-      <c r="B71" s="19">
-        <v>29.65</v>
-      </c>
-      <c r="C71" s="20">
-        <v>2527</v>
-      </c>
-      <c r="D71" s="21">
-        <v>1536</v>
-      </c>
-      <c r="E71" s="21">
-        <v>266</v>
-      </c>
-      <c r="F71" s="21">
-        <v>250</v>
-      </c>
-      <c r="G71" s="22">
-        <f t="shared" si="3"/>
-        <v>1.536</v>
-      </c>
-      <c r="H71" s="22">
-        <f t="shared" si="4"/>
-        <v>0.26600000000000001</v>
-      </c>
-      <c r="I71" s="23">
-        <f t="shared" si="5"/>
-        <v>6.1440000000000001</v>
-      </c>
-      <c r="J71" s="24"/>
+      <c r="B71" s="5">
+        <v>36.46</v>
+      </c>
+      <c r="C71" s="6">
+        <v>2605</v>
+      </c>
+      <c r="D71" s="7">
+        <v>4420</v>
+      </c>
+      <c r="E71" s="7">
+        <v>4380</v>
+      </c>
+      <c r="F71" s="7">
+        <v>3603</v>
+      </c>
+      <c r="G71" s="8">
+        <f t="shared" si="3"/>
+        <v>4.42</v>
+      </c>
+      <c r="H71" s="8">
+        <f t="shared" si="4"/>
+        <v>4.38</v>
+      </c>
+      <c r="I71" s="9">
+        <f t="shared" si="5"/>
+        <v>1.2267554815431585</v>
+      </c>
+      <c r="J71" s="10"/>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="18" t="s">
         <v>79</v>
       </c>
       <c r="B72" s="19">
-        <v>33.869999999999997</v>
+        <v>110.29</v>
       </c>
       <c r="C72" s="20">
-        <v>2696</v>
-      </c>
-      <c r="D72" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="E72" s="25" t="s">
-        <v>80</v>
+        <v>5351</v>
+      </c>
+      <c r="D72" s="21">
+        <v>4395</v>
+      </c>
+      <c r="E72" s="21">
+        <v>616</v>
       </c>
       <c r="F72" s="21">
-        <v>3966</v>
-      </c>
-      <c r="G72" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="H72" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="I72" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="J72" s="28" t="s">
-        <v>82</v>
-      </c>
+        <v>172</v>
+      </c>
+      <c r="G72" s="22">
+        <f t="shared" si="3"/>
+        <v>4.3949999999999996</v>
+      </c>
+      <c r="H72" s="22">
+        <f t="shared" si="4"/>
+        <v>0.61599999999999999</v>
+      </c>
+      <c r="I72" s="23">
+        <f t="shared" si="5"/>
+        <v>25.552325581395348</v>
+      </c>
+      <c r="J72" s="24"/>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="18" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="B73" s="19">
-        <v>39.65</v>
+        <v>29.65</v>
       </c>
       <c r="C73" s="20">
-        <v>2528</v>
-      </c>
-      <c r="D73" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="E73" s="25" t="s">
-        <v>80</v>
+        <v>2527</v>
+      </c>
+      <c r="D73" s="21">
+        <v>1536</v>
+      </c>
+      <c r="E73" s="21">
+        <v>266</v>
       </c>
       <c r="F73" s="21">
-        <v>13714</v>
-      </c>
-      <c r="G73" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="H73" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="I73" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="J73" s="28" t="s">
-        <v>82</v>
-      </c>
+        <v>250</v>
+      </c>
+      <c r="G73" s="22">
+        <f t="shared" si="3"/>
+        <v>1.536</v>
+      </c>
+      <c r="H73" s="22">
+        <f t="shared" si="4"/>
+        <v>0.26600000000000001</v>
+      </c>
+      <c r="I73" s="23">
+        <f t="shared" si="5"/>
+        <v>6.1440000000000001</v>
+      </c>
+      <c r="J73" s="24"/>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B74" s="19">
+        <v>39.65</v>
+      </c>
+      <c r="C74" s="20">
+        <v>2528</v>
+      </c>
+      <c r="D74" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="E74" s="25" t="s">
+        <v>82</v>
+      </c>
+      <c r="F74" s="21">
+        <v>13714</v>
+      </c>
+      <c r="G74" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="H74" s="26" t="s">
+        <v>83</v>
+      </c>
+      <c r="I74" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="J74" s="28" t="s">
         <v>84</v>
-      </c>
-      <c r="B74" s="19">
-        <v>3.24</v>
-      </c>
-      <c r="C74" s="20">
-        <v>1056</v>
-      </c>
-      <c r="D74" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="E74" s="25" t="s">
-        <v>80</v>
-      </c>
-      <c r="F74" s="21">
-        <v>3969</v>
-      </c>
-      <c r="G74" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="H74" s="26" t="s">
-        <v>81</v>
-      </c>
-      <c r="I74" s="27" t="s">
-        <v>81</v>
-      </c>
-      <c r="J74" s="28" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
@@ -3210,7 +3212,7 @@
       </c>
       <c r="I76" s="33">
         <f>IFERROR(AVERAGE(I5:I74),"")</f>
-        <v>3.0564646910026116</v>
+        <v>3.0242352722010546</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
T-06C também usa o ponto de exceção — estrada dele é só interna
O número anterior de T-06C (4,42 km) vinha de uma ligação reta da sede até
um trecho de estrada isolado, que só serve o próprio talhão e não é acesso
real da fazenda. Usuário confirmou e pediu o mesmo ponto de exceção usado
em T-05D/T-CON. Agora T-06C também mostra 7,71 km com o aviso de que a
distância conta a partir de um ponto de acesso confirmado, não de estrada
digitalizada até o talhão.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/FAZENDA_TUCANO_distancias.xlsx
+++ b/FAZENDA_TUCANO_distancias.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\talhoes-distancias\saidas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B788502D-BC5B-4954-BDCD-B4033741965B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EBBB5387-36FD-4F12-B285-30C505E504DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1920" yWindow="1920" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Distâncias" sheetId="1" r:id="rId1"/>
@@ -246,6 +246,9 @@
     <t>T-05D</t>
   </si>
   <si>
+    <t>T-06C</t>
+  </si>
+  <si>
     <t>T-CON</t>
   </si>
   <si>
@@ -268,9 +271,6 @@
   </si>
   <si>
     <t>T-10B</t>
-  </si>
-  <si>
-    <t>T-06C</t>
   </si>
   <si>
     <t>T-01</t>
@@ -2804,10 +2804,10 @@
         <v>70</v>
       </c>
       <c r="B63" s="5">
-        <v>3.24</v>
+        <v>36.46</v>
       </c>
       <c r="C63" s="6">
-        <v>1056</v>
+        <v>2605</v>
       </c>
       <c r="D63" s="7">
         <v>7715</v>
@@ -2816,85 +2816,85 @@
         <v>7715</v>
       </c>
       <c r="F63" s="7">
+        <v>3603</v>
+      </c>
+      <c r="G63" s="8">
+        <f t="shared" si="3"/>
+        <v>7.7149999999999999</v>
+      </c>
+      <c r="H63" s="8">
+        <f t="shared" si="4"/>
+        <v>7.7149999999999999</v>
+      </c>
+      <c r="I63" s="9">
+        <f t="shared" si="5"/>
+        <v>2.1412711629197889</v>
+      </c>
+      <c r="J63" s="10"/>
+    </row>
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A64" s="11" t="s">
+        <v>71</v>
+      </c>
+      <c r="B64" s="12">
+        <v>3.24</v>
+      </c>
+      <c r="C64" s="13">
+        <v>1056</v>
+      </c>
+      <c r="D64" s="14">
+        <v>7715</v>
+      </c>
+      <c r="E64" s="14">
+        <v>7715</v>
+      </c>
+      <c r="F64" s="14">
         <v>3969</v>
       </c>
-      <c r="G63" s="8">
+      <c r="G64" s="15">
         <f t="shared" si="3"/>
         <v>7.7149999999999999</v>
       </c>
-      <c r="H63" s="8">
+      <c r="H64" s="15">
         <f t="shared" si="4"/>
         <v>7.7149999999999999</v>
       </c>
-      <c r="I63" s="9">
+      <c r="I64" s="16">
         <f t="shared" si="5"/>
         <v>1.9438145628621819</v>
       </c>
-      <c r="J63" s="10"/>
-    </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A64" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="B64" s="19">
-        <v>39.74</v>
-      </c>
-      <c r="C64" s="20">
-        <v>3355</v>
-      </c>
-      <c r="D64" s="21">
-        <v>7579</v>
-      </c>
-      <c r="E64" s="21">
-        <v>6617</v>
-      </c>
-      <c r="F64" s="21">
-        <v>1816</v>
-      </c>
-      <c r="G64" s="22">
-        <f t="shared" si="3"/>
-        <v>7.5789999999999997</v>
-      </c>
-      <c r="H64" s="22">
-        <f t="shared" si="4"/>
-        <v>6.617</v>
-      </c>
-      <c r="I64" s="23">
-        <f t="shared" si="5"/>
-        <v>4.1734581497797354</v>
-      </c>
-      <c r="J64" s="24"/>
+      <c r="J64" s="17"/>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="18" t="s">
         <v>72</v>
       </c>
       <c r="B65" s="19">
-        <v>72.52</v>
+        <v>39.74</v>
       </c>
       <c r="C65" s="20">
-        <v>3558</v>
+        <v>3355</v>
       </c>
       <c r="D65" s="21">
-        <v>7432</v>
+        <v>7579</v>
       </c>
       <c r="E65" s="21">
-        <v>6033</v>
+        <v>6617</v>
       </c>
       <c r="F65" s="21">
-        <v>1840</v>
+        <v>1816</v>
       </c>
       <c r="G65" s="22">
         <f t="shared" si="3"/>
-        <v>7.4320000000000004</v>
+        <v>7.5789999999999997</v>
       </c>
       <c r="H65" s="22">
         <f t="shared" si="4"/>
-        <v>6.0330000000000004</v>
+        <v>6.617</v>
       </c>
       <c r="I65" s="23">
         <f t="shared" si="5"/>
-        <v>4.0391304347826091</v>
+        <v>4.1734581497797354</v>
       </c>
       <c r="J65" s="24"/>
     </row>
@@ -2903,31 +2903,31 @@
         <v>73</v>
       </c>
       <c r="B66" s="19">
-        <v>93.41</v>
+        <v>72.52</v>
       </c>
       <c r="C66" s="20">
-        <v>4212</v>
+        <v>3558</v>
       </c>
       <c r="D66" s="21">
-        <v>6651</v>
+        <v>7432</v>
       </c>
       <c r="E66" s="21">
-        <v>5303</v>
+        <v>6033</v>
       </c>
       <c r="F66" s="21">
-        <v>539</v>
+        <v>1840</v>
       </c>
       <c r="G66" s="22">
         <f t="shared" si="3"/>
-        <v>6.6509999999999998</v>
+        <v>7.4320000000000004</v>
       </c>
       <c r="H66" s="22">
         <f t="shared" si="4"/>
-        <v>5.3029999999999999</v>
+        <v>6.0330000000000004</v>
       </c>
       <c r="I66" s="23">
         <f t="shared" si="5"/>
-        <v>12.339517625231911</v>
+        <v>4.0391304347826091</v>
       </c>
       <c r="J66" s="24"/>
     </row>
@@ -2936,31 +2936,31 @@
         <v>74</v>
       </c>
       <c r="B67" s="19">
-        <v>30.12</v>
+        <v>93.41</v>
       </c>
       <c r="C67" s="20">
-        <v>2592</v>
+        <v>4212</v>
       </c>
       <c r="D67" s="21">
-        <v>6617</v>
+        <v>6651</v>
       </c>
       <c r="E67" s="21">
-        <v>5688</v>
+        <v>5303</v>
       </c>
       <c r="F67" s="21">
-        <v>929</v>
+        <v>539</v>
       </c>
       <c r="G67" s="22">
         <f t="shared" si="3"/>
-        <v>6.617</v>
+        <v>6.6509999999999998</v>
       </c>
       <c r="H67" s="22">
         <f t="shared" si="4"/>
-        <v>5.6879999999999997</v>
+        <v>5.3029999999999999</v>
       </c>
       <c r="I67" s="23">
         <f t="shared" si="5"/>
-        <v>7.1227125941872984</v>
+        <v>12.339517625231911</v>
       </c>
       <c r="J67" s="24"/>
     </row>
@@ -2969,31 +2969,31 @@
         <v>75</v>
       </c>
       <c r="B68" s="19">
-        <v>159.81</v>
+        <v>30.12</v>
       </c>
       <c r="C68" s="20">
-        <v>5989</v>
+        <v>2592</v>
       </c>
       <c r="D68" s="21">
-        <v>6061</v>
+        <v>6617</v>
       </c>
       <c r="E68" s="21">
-        <v>3243</v>
+        <v>5688</v>
       </c>
       <c r="F68" s="21">
-        <v>623</v>
+        <v>929</v>
       </c>
       <c r="G68" s="22">
         <f t="shared" si="3"/>
-        <v>6.0609999999999999</v>
+        <v>6.617</v>
       </c>
       <c r="H68" s="22">
         <f t="shared" si="4"/>
-        <v>3.2429999999999999</v>
+        <v>5.6879999999999997</v>
       </c>
       <c r="I68" s="23">
         <f t="shared" si="5"/>
-        <v>9.728731942215088</v>
+        <v>7.1227125941872984</v>
       </c>
       <c r="J68" s="24"/>
     </row>
@@ -3002,31 +3002,31 @@
         <v>76</v>
       </c>
       <c r="B69" s="19">
-        <v>226.37</v>
+        <v>159.81</v>
       </c>
       <c r="C69" s="20">
-        <v>7413</v>
+        <v>5989</v>
       </c>
       <c r="D69" s="21">
-        <v>6005</v>
+        <v>6061</v>
       </c>
       <c r="E69" s="21">
-        <v>3122</v>
+        <v>3243</v>
       </c>
       <c r="F69" s="21">
-        <v>554</v>
+        <v>623</v>
       </c>
       <c r="G69" s="22">
         <f t="shared" si="3"/>
-        <v>6.0049999999999999</v>
+        <v>6.0609999999999999</v>
       </c>
       <c r="H69" s="22">
         <f t="shared" si="4"/>
-        <v>3.1219999999999999</v>
+        <v>3.2429999999999999</v>
       </c>
       <c r="I69" s="23">
         <f t="shared" si="5"/>
-        <v>10.839350180505415</v>
+        <v>9.728731942215088</v>
       </c>
       <c r="J69" s="24"/>
     </row>
@@ -3035,66 +3035,66 @@
         <v>77</v>
       </c>
       <c r="B70" s="19">
+        <v>226.37</v>
+      </c>
+      <c r="C70" s="20">
+        <v>7413</v>
+      </c>
+      <c r="D70" s="21">
+        <v>6005</v>
+      </c>
+      <c r="E70" s="21">
+        <v>3122</v>
+      </c>
+      <c r="F70" s="21">
+        <v>554</v>
+      </c>
+      <c r="G70" s="22">
+        <f t="shared" si="3"/>
+        <v>6.0049999999999999</v>
+      </c>
+      <c r="H70" s="22">
+        <f t="shared" si="4"/>
+        <v>3.1219999999999999</v>
+      </c>
+      <c r="I70" s="23">
+        <f t="shared" si="5"/>
+        <v>10.839350180505415</v>
+      </c>
+      <c r="J70" s="24"/>
+    </row>
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A71" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="B71" s="19">
         <v>127.8</v>
       </c>
-      <c r="C70" s="20">
+      <c r="C71" s="20">
         <v>5228</v>
       </c>
-      <c r="D70" s="21">
+      <c r="D71" s="21">
         <v>5303</v>
       </c>
-      <c r="E70" s="21">
+      <c r="E71" s="21">
         <v>1483</v>
       </c>
-      <c r="F70" s="21">
+      <c r="F71" s="21">
         <v>289</v>
       </c>
-      <c r="G70" s="22">
+      <c r="G71" s="22">
         <f t="shared" si="3"/>
         <v>5.3029999999999999</v>
       </c>
-      <c r="H70" s="22">
+      <c r="H71" s="22">
         <f t="shared" si="4"/>
         <v>1.4830000000000001</v>
       </c>
-      <c r="I70" s="23">
+      <c r="I71" s="23">
         <f t="shared" si="5"/>
         <v>18.349480968858131</v>
       </c>
-      <c r="J70" s="24"/>
-    </row>
-    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
-      <c r="A71" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="B71" s="5">
-        <v>36.46</v>
-      </c>
-      <c r="C71" s="6">
-        <v>2605</v>
-      </c>
-      <c r="D71" s="7">
-        <v>4420</v>
-      </c>
-      <c r="E71" s="7">
-        <v>4380</v>
-      </c>
-      <c r="F71" s="7">
-        <v>3603</v>
-      </c>
-      <c r="G71" s="8">
-        <f t="shared" si="3"/>
-        <v>4.42</v>
-      </c>
-      <c r="H71" s="8">
-        <f t="shared" si="4"/>
-        <v>4.38</v>
-      </c>
-      <c r="I71" s="9">
-        <f t="shared" si="5"/>
-        <v>1.2267554815431585</v>
-      </c>
-      <c r="J71" s="10"/>
+      <c r="J71" s="24"/>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="18" t="s">
@@ -3212,7 +3212,7 @@
       </c>
       <c r="I76" s="33">
         <f>IFERROR(AVERAGE(I5:I74),"")</f>
-        <v>3.0242352722010546</v>
+        <v>3.0374891226557881</v>
       </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">

</xml_diff>